<commit_message>
Update project until august 2024
</commit_message>
<xml_diff>
--- a/00_overall_data/som_admin2.xlsx
+++ b/00_overall_data/som_admin2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="26626"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27126"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lshtm-my.sharepoint.com/personal/lshyo5_lshtm_ac_uk/Documents/Documents/GitHub/ME_Somalia/overall_data/data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://lshtm-my.sharepoint.com/personal/lshyo5_lshtm_ac_uk/Documents/Documents/GitHub/mortality_estimation/00_overall_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="128" documentId="13_ncr:1_{DECFC3CA-D1B0-4903-844A-C514355A3AD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{736DB2EC-102F-40D2-A315-C2CDE9D56DE8}"/>
+  <xr:revisionPtr revIDLastSave="131" documentId="13_ncr:1_{DECFC3CA-D1B0-4903-844A-C514355A3AD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0556D27E-8FB1-417C-92F8-2B2A04D47FB8}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="strata" sheetId="51" r:id="rId1"/>
@@ -19,7 +19,7 @@
     <externalReference r:id="rId2"/>
   </externalReferences>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">strata!$A$1:$C$66</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">strata!$A$1:$E$75</definedName>
     <definedName name="admin1">strata!$B:$B</definedName>
     <definedName name="causal_level">#REF!</definedName>
     <definedName name="domain">#REF!</definedName>
@@ -638,10 +638,6 @@
 </externalLink>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
@@ -906,15 +902,15 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:E75"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="20.42578125" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.85546875" style="2" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.140625" style="2" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.44140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="15.88671875" style="2" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.109375" style="2" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -931,7 +927,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>3</v>
       </c>
@@ -948,7 +944,7 @@
         <v>1102</v>
       </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>3</v>
       </c>
@@ -965,7 +961,7 @@
         <v>1101</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -982,7 +978,7 @@
         <v>1103</v>
       </c>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
         <v>3</v>
       </c>
@@ -999,7 +995,7 @@
         <v>1104</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
         <v>3</v>
       </c>
@@ -1016,7 +1012,7 @@
         <v>1602</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>3</v>
       </c>
@@ -1033,7 +1029,7 @@
         <v>1601</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
         <v>3</v>
       </c>
@@ -1050,7 +1046,7 @@
         <v>1603</v>
       </c>
     </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
         <v>3</v>
       </c>
@@ -1067,7 +1063,7 @@
         <v>1604</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
         <v>3</v>
       </c>
@@ -1084,7 +1080,7 @@
         <v>1605</v>
       </c>
     </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
         <v>3</v>
       </c>
@@ -1101,7 +1097,7 @@
         <v>1606</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>3</v>
       </c>
@@ -1118,7 +1114,7 @@
         <v>1801</v>
       </c>
     </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="3" t="s">
         <v>3</v>
       </c>
@@ -1135,7 +1131,7 @@
         <v>1802</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="3" t="s">
         <v>3</v>
       </c>
@@ -1152,7 +1148,7 @@
         <v>1803</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="3" t="s">
         <v>3</v>
       </c>
@@ -1169,7 +1165,7 @@
         <v>1804</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="3" t="s">
         <v>3</v>
       </c>
@@ -1186,7 +1182,7 @@
         <v>1805</v>
       </c>
     </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="3" t="s">
         <v>3</v>
       </c>
@@ -1203,7 +1199,7 @@
         <v>1702</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="3" t="s">
         <v>3</v>
       </c>
@@ -1220,7 +1216,7 @@
         <v>1703</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="3" t="s">
         <v>3</v>
       </c>
@@ -1237,7 +1233,7 @@
         <v>1701</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="3" t="s">
         <v>3</v>
       </c>
@@ -1254,7 +1250,7 @@
         <v>1502</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
         <v>3</v>
       </c>
@@ -1271,7 +1267,7 @@
         <v>1501</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
         <v>3</v>
       </c>
@@ -1288,7 +1284,7 @@
         <v>1503</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
         <v>3</v>
       </c>
@@ -1305,7 +1301,7 @@
         <v>1402</v>
       </c>
     </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
         <v>3</v>
       </c>
@@ -1322,7 +1318,7 @@
         <v>1401</v>
       </c>
     </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
         <v>3</v>
       </c>
@@ -1339,7 +1335,7 @@
         <v>1403</v>
       </c>
     </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
         <v>3</v>
       </c>
@@ -1356,7 +1352,7 @@
         <v>1404</v>
       </c>
     </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
         <v>3</v>
       </c>
@@ -1373,7 +1369,7 @@
         <v>1301</v>
       </c>
     </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
         <v>3</v>
       </c>
@@ -1390,7 +1386,7 @@
         <v>1302</v>
       </c>
     </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
         <v>3</v>
       </c>
@@ -1407,7 +1403,7 @@
         <v>1303</v>
       </c>
     </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
         <v>3</v>
       </c>
@@ -1424,7 +1420,7 @@
         <v>1304</v>
       </c>
     </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
         <v>3</v>
       </c>
@@ -1441,7 +1437,7 @@
         <v>1202</v>
       </c>
     </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
         <v>3</v>
       </c>
@@ -1458,7 +1454,7 @@
         <v>1203</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
         <v>3</v>
       </c>
@@ -1475,7 +1471,7 @@
         <v>1201</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="3" t="s">
         <v>44</v>
       </c>
@@ -1492,7 +1488,7 @@
         <v>2502</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
         <v>44</v>
       </c>
@@ -1509,7 +1505,7 @@
         <v>2505</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
         <v>44</v>
       </c>
@@ -1526,7 +1522,7 @@
         <v>2503</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
         <v>44</v>
       </c>
@@ -1543,7 +1539,7 @@
         <v>2504</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
         <v>44</v>
       </c>
@@ -1560,7 +1556,7 @@
         <v>2501</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="3" t="s">
         <v>44</v>
       </c>
@@ -1577,7 +1573,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
         <v>44</v>
       </c>
@@ -1594,7 +1590,7 @@
         <v>2401</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
         <v>44</v>
       </c>
@@ -1611,7 +1607,7 @@
         <v>2402</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="3" t="s">
         <v>44</v>
       </c>
@@ -1628,7 +1624,7 @@
         <v>2403</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
         <v>44</v>
       </c>
@@ -1645,7 +1641,7 @@
         <v>2404</v>
       </c>
     </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
         <v>44</v>
       </c>
@@ -1662,7 +1658,7 @@
         <v>1902</v>
       </c>
     </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="3" t="s">
         <v>44</v>
       </c>
@@ -1679,7 +1675,7 @@
         <v>1903</v>
       </c>
     </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="3" t="s">
         <v>44</v>
       </c>
@@ -1696,7 +1692,7 @@
         <v>1904</v>
       </c>
     </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
         <v>44</v>
       </c>
@@ -1713,7 +1709,7 @@
         <v>1905</v>
       </c>
     </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
         <v>44</v>
       </c>
@@ -1730,7 +1726,7 @@
         <v>1901</v>
       </c>
     </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
         <v>44</v>
       </c>
@@ -1747,7 +1743,7 @@
         <v>2602</v>
       </c>
     </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="3" t="s">
         <v>44</v>
       </c>
@@ -1764,7 +1760,7 @@
         <v>2603</v>
       </c>
     </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
         <v>44</v>
       </c>
@@ -1781,7 +1777,7 @@
         <v>2604</v>
       </c>
     </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="3" t="s">
         <v>44</v>
       </c>
@@ -1798,7 +1794,7 @@
         <v>2605</v>
       </c>
     </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" s="3" t="s">
         <v>44</v>
       </c>
@@ -1815,7 +1811,7 @@
         <v>2601</v>
       </c>
     </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A54" s="3" t="s">
         <v>44</v>
       </c>
@@ -1832,7 +1828,7 @@
         <v>2606</v>
       </c>
     </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" s="3" t="s">
         <v>44</v>
       </c>
@@ -1849,7 +1845,7 @@
         <v>2001</v>
       </c>
     </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="3" t="s">
         <v>44</v>
       </c>
@@ -1866,7 +1862,7 @@
         <v>2002</v>
       </c>
     </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
         <v>44</v>
       </c>
@@ -1883,7 +1879,7 @@
         <v>2003</v>
       </c>
     </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" s="3" t="s">
         <v>44</v>
       </c>
@@ -1900,7 +1896,7 @@
         <v>2802</v>
       </c>
     </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="3" t="s">
         <v>44</v>
       </c>
@@ -1917,7 +1913,7 @@
         <v>2803</v>
       </c>
     </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" s="3" t="s">
         <v>44</v>
       </c>
@@ -1934,7 +1930,7 @@
         <v>2804</v>
       </c>
     </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" s="3" t="s">
         <v>44</v>
       </c>
@@ -1951,7 +1947,7 @@
         <v>2801</v>
       </c>
     </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" s="3" t="s">
         <v>44</v>
       </c>
@@ -1968,7 +1964,7 @@
         <v>2302</v>
       </c>
     </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" s="3" t="s">
         <v>44</v>
       </c>
@@ -1985,7 +1981,7 @@
         <v>2303</v>
       </c>
     </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" s="3" t="s">
         <v>44</v>
       </c>
@@ -2002,7 +1998,7 @@
         <v>2304</v>
       </c>
     </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" s="3" t="s">
         <v>44</v>
       </c>
@@ -2019,7 +2015,7 @@
         <v>2301</v>
       </c>
     </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" s="3" t="s">
         <v>44</v>
       </c>
@@ -2036,7 +2032,7 @@
         <v>2305</v>
       </c>
     </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" s="3" t="s">
         <v>44</v>
       </c>
@@ -2053,7 +2049,7 @@
         <v>2306</v>
       </c>
     </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" s="3" t="s">
         <v>44</v>
       </c>
@@ -2070,7 +2066,7 @@
         <v>2307</v>
       </c>
     </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" s="3" t="s">
         <v>44</v>
       </c>
@@ -2087,7 +2083,7 @@
         <v>2701</v>
       </c>
     </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" s="3" t="s">
         <v>44</v>
       </c>
@@ -2104,7 +2100,7 @@
         <v>2702</v>
       </c>
     </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" s="3" t="s">
         <v>44</v>
       </c>
@@ -2121,7 +2117,7 @@
         <v>2703</v>
       </c>
     </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" s="3" t="s">
         <v>44</v>
       </c>
@@ -2138,7 +2134,7 @@
         <v>2102</v>
       </c>
     </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" s="3" t="s">
         <v>44</v>
       </c>
@@ -2155,7 +2151,7 @@
         <v>2103</v>
       </c>
     </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" s="3" t="s">
         <v>44</v>
       </c>
@@ -2172,7 +2168,7 @@
         <v>2104</v>
       </c>
     </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A75" s="3" t="s">
         <v>44</v>
       </c>
@@ -2190,6 +2186,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E75" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:C66">
     <sortCondition ref="A2:A66"/>
     <sortCondition ref="C2:C66"/>

</xml_diff>